<commit_message>
Dynamic Excel sheet viewer 100 percent
</commit_message>
<xml_diff>
--- a/distribution_live_backup.xlsx
+++ b/distribution_live_backup.xlsx
@@ -6411,16 +6411,7 @@
         <v>Given</v>
       </c>
       <c r="G258" t="str">
-        <v>Ilyas</v>
-      </c>
-      <c r="H258" t="str">
-        <v>17/05/2026</v>
-      </c>
-      <c r="I258" t="str">
-        <v>Sunday</v>
-      </c>
-      <c r="J258" t="str">
-        <v>16:00:54</v>
+        <v/>
       </c>
     </row>
     <row r="259">

</xml_diff>